<commit_message>
football_odds: half-time layer — HT score, FT score and HT/FT combination for analogues
- outcome_stats: half-time result shares and the 9-way HT/FT distribution
  (rows without a half-time result excluded from that layer only)
- analogue export carries ht_score and htft ('1/1', 'X/2', ...); details JSON
  and API expose them; frontend shows İlk yarı / Maç sonu / İY/MS columns in the
  analogue list plus an HT/FT distribution section and glossary entry

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EGUrFNWpQmRQCkeHWoEgSz
</commit_message>
<xml_diff>
--- a/football_odds/results/2026-09-14_predictions.xlsx
+++ b/football_odds/results/2026-09-14_predictions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CO12"/>
+  <dimension ref="A1:CS12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -844,40 +844,60 @@
       </c>
       <c r="CH1" t="inlineStr">
         <is>
+          <t>ht_h</t>
+        </is>
+      </c>
+      <c r="CI1" t="inlineStr">
+        <is>
+          <t>ht_d</t>
+        </is>
+      </c>
+      <c r="CJ1" t="inlineStr">
+        <is>
+          <t>ht_a</t>
+        </is>
+      </c>
+      <c r="CK1" t="inlineStr">
+        <is>
+          <t>n_ht</t>
+        </is>
+      </c>
+      <c r="CL1" t="inlineStr">
+        <is>
           <t>tol_probs_1pct</t>
         </is>
       </c>
-      <c r="CI1" t="inlineStr">
+      <c r="CM1" t="inlineStr">
         <is>
           <t>tol_probs_2pct</t>
         </is>
       </c>
-      <c r="CJ1" t="inlineStr">
+      <c r="CN1" t="inlineStr">
         <is>
           <t>tol_probs_3pct</t>
         </is>
       </c>
-      <c r="CK1" t="inlineStr">
+      <c r="CO1" t="inlineStr">
         <is>
           <t>tol_probs_5pct</t>
         </is>
       </c>
-      <c r="CL1" t="inlineStr">
+      <c r="CP1" t="inlineStr">
         <is>
           <t>tol_odds_1pct</t>
         </is>
       </c>
-      <c r="CM1" t="inlineStr">
+      <c r="CQ1" t="inlineStr">
         <is>
           <t>tol_odds_2pct</t>
         </is>
       </c>
-      <c r="CN1" t="inlineStr">
+      <c r="CR1" t="inlineStr">
         <is>
           <t>tol_odds_3pct</t>
         </is>
       </c>
-      <c r="CO1" t="inlineStr">
+      <c r="CS1" t="inlineStr">
         <is>
           <t>tol_odds_5pct</t>
         </is>
@@ -1164,27 +1184,39 @@
         <v>98.896</v>
       </c>
       <c r="CH2" t="n">
+        <v>62</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>30</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>8</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>500</v>
+      </c>
+      <c r="CL2" t="n">
         <v>349</v>
       </c>
-      <c r="CI2" t="n">
+      <c r="CM2" t="n">
         <v>1229</v>
       </c>
-      <c r="CJ2" t="n">
+      <c r="CN2" t="n">
         <v>2084</v>
       </c>
-      <c r="CK2" t="n">
+      <c r="CO2" t="n">
         <v>3459</v>
       </c>
-      <c r="CL2" t="n">
+      <c r="CP2" t="n">
         <v>3</v>
       </c>
-      <c r="CM2" t="n">
+      <c r="CQ2" t="n">
         <v>13</v>
       </c>
-      <c r="CN2" t="n">
+      <c r="CR2" t="n">
         <v>38</v>
       </c>
-      <c r="CO2" t="n">
+      <c r="CS2" t="n">
         <v>128</v>
       </c>
     </row>
@@ -1469,27 +1501,39 @@
         <v>98.786</v>
       </c>
       <c r="CH3" t="n">
+        <v>14.83</v>
+      </c>
+      <c r="CI3" t="n">
+        <v>40.08</v>
+      </c>
+      <c r="CJ3" t="n">
+        <v>45.09</v>
+      </c>
+      <c r="CK3" t="n">
+        <v>499</v>
+      </c>
+      <c r="CL3" t="n">
         <v>265</v>
       </c>
-      <c r="CI3" t="n">
+      <c r="CM3" t="n">
         <v>969</v>
       </c>
-      <c r="CJ3" t="n">
+      <c r="CN3" t="n">
         <v>1674</v>
       </c>
-      <c r="CK3" t="n">
+      <c r="CO3" t="n">
         <v>3021</v>
       </c>
-      <c r="CL3" t="n">
+      <c r="CP3" t="n">
         <v>5</v>
       </c>
-      <c r="CM3" t="n">
+      <c r="CQ3" t="n">
         <v>32</v>
       </c>
-      <c r="CN3" t="n">
+      <c r="CR3" t="n">
         <v>98</v>
       </c>
-      <c r="CO3" t="n">
+      <c r="CS3" t="n">
         <v>299</v>
       </c>
     </row>
@@ -1774,27 +1818,39 @@
         <v>98.372</v>
       </c>
       <c r="CH4" t="n">
+        <v>15.462</v>
+      </c>
+      <c r="CI4" t="n">
+        <v>39.558</v>
+      </c>
+      <c r="CJ4" t="n">
+        <v>44.98</v>
+      </c>
+      <c r="CK4" t="n">
+        <v>498</v>
+      </c>
+      <c r="CL4" t="n">
         <v>280</v>
       </c>
-      <c r="CI4" t="n">
+      <c r="CM4" t="n">
         <v>944</v>
       </c>
-      <c r="CJ4" t="n">
+      <c r="CN4" t="n">
         <v>1702</v>
       </c>
-      <c r="CK4" t="n">
+      <c r="CO4" t="n">
         <v>3104</v>
       </c>
-      <c r="CL4" t="n">
+      <c r="CP4" t="n">
         <v>0</v>
       </c>
-      <c r="CM4" t="n">
+      <c r="CQ4" t="n">
         <v>6</v>
       </c>
-      <c r="CN4" t="n">
+      <c r="CR4" t="n">
         <v>15</v>
       </c>
-      <c r="CO4" t="n">
+      <c r="CS4" t="n">
         <v>143</v>
       </c>
     </row>
@@ -2079,27 +2135,39 @@
         <v>99.384</v>
       </c>
       <c r="CH5" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="CI5" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="CJ5" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="CK5" t="n">
+        <v>500</v>
+      </c>
+      <c r="CL5" t="n">
         <v>1126</v>
       </c>
-      <c r="CI5" t="n">
+      <c r="CM5" t="n">
         <v>3873</v>
       </c>
-      <c r="CJ5" t="n">
+      <c r="CN5" t="n">
         <v>7536</v>
       </c>
-      <c r="CK5" t="n">
+      <c r="CO5" t="n">
         <v>15240</v>
       </c>
-      <c r="CL5" t="n">
+      <c r="CP5" t="n">
         <v>3</v>
       </c>
-      <c r="CM5" t="n">
+      <c r="CQ5" t="n">
         <v>64</v>
       </c>
-      <c r="CN5" t="n">
+      <c r="CR5" t="n">
         <v>336</v>
       </c>
-      <c r="CO5" t="n">
+      <c r="CS5" t="n">
         <v>1482</v>
       </c>
     </row>
@@ -2384,27 +2452,39 @@
         <v>98.961</v>
       </c>
       <c r="CH6" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="CI6" t="n">
+        <v>43.4</v>
+      </c>
+      <c r="CJ6" t="n">
+        <v>35</v>
+      </c>
+      <c r="CK6" t="n">
+        <v>500</v>
+      </c>
+      <c r="CL6" t="n">
         <v>544</v>
       </c>
-      <c r="CI6" t="n">
+      <c r="CM6" t="n">
         <v>2123</v>
       </c>
-      <c r="CJ6" t="n">
+      <c r="CN6" t="n">
         <v>4431</v>
       </c>
-      <c r="CK6" t="n">
+      <c r="CO6" t="n">
         <v>9576</v>
       </c>
-      <c r="CL6" t="n">
+      <c r="CP6" t="n">
         <v>6</v>
       </c>
-      <c r="CM6" t="n">
+      <c r="CQ6" t="n">
         <v>41</v>
       </c>
-      <c r="CN6" t="n">
+      <c r="CR6" t="n">
         <v>125</v>
       </c>
-      <c r="CO6" t="n">
+      <c r="CS6" t="n">
         <v>597</v>
       </c>
     </row>
@@ -2689,27 +2769,39 @@
         <v>98.82899999999999</v>
       </c>
       <c r="CH7" t="n">
+        <v>27</v>
+      </c>
+      <c r="CI7" t="n">
+        <v>44</v>
+      </c>
+      <c r="CJ7" t="n">
+        <v>29</v>
+      </c>
+      <c r="CK7" t="n">
+        <v>500</v>
+      </c>
+      <c r="CL7" t="n">
         <v>1102</v>
       </c>
-      <c r="CI7" t="n">
+      <c r="CM7" t="n">
         <v>3925</v>
       </c>
-      <c r="CJ7" t="n">
+      <c r="CN7" t="n">
         <v>8026</v>
       </c>
-      <c r="CK7" t="n">
+      <c r="CO7" t="n">
         <v>17168</v>
       </c>
-      <c r="CL7" t="n">
+      <c r="CP7" t="n">
         <v>2</v>
       </c>
-      <c r="CM7" t="n">
+      <c r="CQ7" t="n">
         <v>50</v>
       </c>
-      <c r="CN7" t="n">
+      <c r="CR7" t="n">
         <v>172</v>
       </c>
-      <c r="CO7" t="n">
+      <c r="CS7" t="n">
         <v>1039</v>
       </c>
     </row>
@@ -2994,27 +3086,39 @@
         <v>99.148</v>
       </c>
       <c r="CH8" t="n">
+        <v>57.715</v>
+      </c>
+      <c r="CI8" t="n">
+        <v>32.265</v>
+      </c>
+      <c r="CJ8" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="CK8" t="n">
+        <v>499</v>
+      </c>
+      <c r="CL8" t="n">
         <v>545</v>
       </c>
-      <c r="CI8" t="n">
+      <c r="CM8" t="n">
         <v>1403</v>
       </c>
-      <c r="CJ8" t="n">
+      <c r="CN8" t="n">
         <v>2173</v>
       </c>
-      <c r="CK8" t="n">
+      <c r="CO8" t="n">
         <v>3774</v>
       </c>
-      <c r="CL8" t="n">
+      <c r="CP8" t="n">
         <v>5</v>
       </c>
-      <c r="CM8" t="n">
+      <c r="CQ8" t="n">
         <v>27</v>
       </c>
-      <c r="CN8" t="n">
+      <c r="CR8" t="n">
         <v>89</v>
       </c>
-      <c r="CO8" t="n">
+      <c r="CS8" t="n">
         <v>274</v>
       </c>
     </row>
@@ -3299,27 +3403,39 @@
         <v>99.199</v>
       </c>
       <c r="CH9" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="CI9" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="CJ9" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="CK9" t="n">
+        <v>500</v>
+      </c>
+      <c r="CL9" t="n">
         <v>717</v>
       </c>
-      <c r="CI9" t="n">
+      <c r="CM9" t="n">
         <v>3424</v>
       </c>
-      <c r="CJ9" t="n">
+      <c r="CN9" t="n">
         <v>7530</v>
       </c>
-      <c r="CK9" t="n">
+      <c r="CO9" t="n">
         <v>18467</v>
       </c>
-      <c r="CL9" t="n">
+      <c r="CP9" t="n">
         <v>26</v>
       </c>
-      <c r="CM9" t="n">
+      <c r="CQ9" t="n">
         <v>149</v>
       </c>
-      <c r="CN9" t="n">
+      <c r="CR9" t="n">
         <v>486</v>
       </c>
-      <c r="CO9" t="n">
+      <c r="CS9" t="n">
         <v>1780</v>
       </c>
     </row>
@@ -3604,27 +3720,39 @@
         <v>98.66500000000001</v>
       </c>
       <c r="CH10" t="n">
+        <v>44</v>
+      </c>
+      <c r="CI10" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="CJ10" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="CK10" t="n">
+        <v>500</v>
+      </c>
+      <c r="CL10" t="n">
         <v>234</v>
       </c>
-      <c r="CI10" t="n">
+      <c r="CM10" t="n">
         <v>1239</v>
       </c>
-      <c r="CJ10" t="n">
+      <c r="CN10" t="n">
         <v>3798</v>
       </c>
-      <c r="CK10" t="n">
+      <c r="CO10" t="n">
         <v>14083</v>
       </c>
-      <c r="CL10" t="n">
+      <c r="CP10" t="n">
         <v>0</v>
       </c>
-      <c r="CM10" t="n">
+      <c r="CQ10" t="n">
         <v>21</v>
       </c>
-      <c r="CN10" t="n">
+      <c r="CR10" t="n">
         <v>87</v>
       </c>
-      <c r="CO10" t="n">
+      <c r="CS10" t="n">
         <v>468</v>
       </c>
     </row>
@@ -3909,27 +4037,39 @@
         <v>99.518</v>
       </c>
       <c r="CH11" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="CI11" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="CJ11" t="n">
+        <v>25</v>
+      </c>
+      <c r="CK11" t="n">
+        <v>500</v>
+      </c>
+      <c r="CL11" t="n">
         <v>1849</v>
       </c>
-      <c r="CI11" t="n">
+      <c r="CM11" t="n">
         <v>6327</v>
       </c>
-      <c r="CJ11" t="n">
+      <c r="CN11" t="n">
         <v>11451</v>
       </c>
-      <c r="CK11" t="n">
+      <c r="CO11" t="n">
         <v>21181</v>
       </c>
-      <c r="CL11" t="n">
+      <c r="CP11" t="n">
         <v>19</v>
       </c>
-      <c r="CM11" t="n">
+      <c r="CQ11" t="n">
         <v>175</v>
       </c>
-      <c r="CN11" t="n">
+      <c r="CR11" t="n">
         <v>680</v>
       </c>
-      <c r="CO11" t="n">
+      <c r="CS11" t="n">
         <v>2741</v>
       </c>
     </row>
@@ -4214,27 +4354,39 @@
         <v>99.036</v>
       </c>
       <c r="CH12" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="CI12" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="CJ12" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="CK12" t="n">
+        <v>500</v>
+      </c>
+      <c r="CL12" t="n">
         <v>623</v>
       </c>
-      <c r="CI12" t="n">
+      <c r="CM12" t="n">
         <v>2181</v>
       </c>
-      <c r="CJ12" t="n">
+      <c r="CN12" t="n">
         <v>3864</v>
       </c>
-      <c r="CK12" t="n">
+      <c r="CO12" t="n">
         <v>6943</v>
       </c>
-      <c r="CL12" t="n">
+      <c r="CP12" t="n">
         <v>4</v>
       </c>
-      <c r="CM12" t="n">
+      <c r="CQ12" t="n">
         <v>19</v>
       </c>
-      <c r="CN12" t="n">
+      <c r="CR12" t="n">
         <v>104</v>
       </c>
-      <c r="CO12" t="n">
+      <c r="CS12" t="n">
         <v>545</v>
       </c>
     </row>

</xml_diff>